<commit_message>
Link spreadsheet exercises to free Excel on the web.
Open each cotacao/PROCV/decision pack in Microsoft Excel Online via Office viewer links, while keeping the on-site sheet as a fallback.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/exercicios/treino-compras-01-cotacao.xlsx
+++ b/public/exercicios/treino-compras-01-cotacao.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="60">
   <si>
     <t>TREINO COMPRAS — Exercício 1: Cotação</t>
   </si>
@@ -22,7 +22,7 @@
     <t/>
   </si>
   <si>
-    <t>Objetivo: praticar fórmulas no Excel de verdade.</t>
+    <t>Objetivo: praticar fórmulas no Excel na Web.</t>
   </si>
   <si>
     <t>1) Vá para a aba Cotacao</t>
@@ -40,10 +40,7 @@
     <t>5) Coluna L (Melhor): =MÍNIMO(J2:K2)  ou  =MIN(J2:K2)</t>
   </si>
   <si>
-    <t>6) Salve como .xlsx e envie no site para corrigir</t>
-  </si>
-  <si>
-    <t>Dica Google Sheets: Arquivo &gt; Fazer download &gt; Microsoft Excel (.xlsx)</t>
+    <t>6) Se abriu só em visualização, use Editar no navegador / Salvar uma cópia</t>
   </si>
   <si>
     <t>Produto</t>
@@ -826,9 +823,7 @@
       <c r="P10" s="2"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -846,9 +841,7 @@
       <c r="P11" s="2"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -1571,40 +1564,40 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
@@ -1613,16 +1606,16 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C2" s="2">
         <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2">
         <v>0.95</v>
@@ -1631,7 +1624,7 @@
         <v>25</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H2" s="2">
         <v>1.1</v>
@@ -1649,16 +1642,16 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="C3" s="2">
         <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2">
         <v>0.18</v>
@@ -1667,7 +1660,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H3" s="2">
         <v>0.15</v>
@@ -1685,16 +1678,16 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="C4" s="2">
         <v>50</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" s="2">
         <v>8</v>
@@ -1703,7 +1696,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H4" s="2">
         <v>7.2</v>
@@ -1721,16 +1714,16 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="C5" s="2">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" s="2">
         <v>12.5</v>
@@ -1739,7 +1732,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H5" s="2">
         <v>14</v>
@@ -1757,16 +1750,16 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="C6" s="2">
         <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2">
         <v>34</v>
@@ -1775,7 +1768,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H6" s="2">
         <v>31</v>
@@ -1793,16 +1786,16 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="C7" s="2">
         <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" s="2">
         <v>2.5</v>
@@ -1811,7 +1804,7 @@
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H7" s="2">
         <v>2.8</v>
@@ -1829,16 +1822,16 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="C8" s="2">
         <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E8" s="2">
         <v>4.2</v>
@@ -1847,7 +1840,7 @@
         <v>18</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H8" s="2">
         <v>3.9</v>
@@ -1865,16 +1858,16 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2">
         <v>280</v>
@@ -1883,7 +1876,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H9" s="2">
         <v>265</v>
@@ -1901,16 +1894,16 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="2">
         <v>45</v>
@@ -1919,7 +1912,7 @@
         <v>22</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H10" s="2">
         <v>48</v>
@@ -1937,16 +1930,16 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11" s="2">
         <v>32</v>
@@ -1955,7 +1948,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H11" s="2">
         <v>29</v>
@@ -2690,7 +2683,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2710,10 +2703,10 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2732,10 +2725,10 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -2754,10 +2747,10 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2796,7 +2789,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -3619,40 +3612,40 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
@@ -3661,16 +3654,16 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C2" s="2">
         <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2">
         <v>0.95</v>
@@ -3679,7 +3672,7 @@
         <v>25</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H2" s="2">
         <v>1.1</v>
@@ -3703,16 +3696,16 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="C3" s="2">
         <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2">
         <v>0.18</v>
@@ -3721,7 +3714,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H3" s="2">
         <v>0.15</v>
@@ -3745,16 +3738,16 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="C4" s="2">
         <v>50</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" s="2">
         <v>8</v>
@@ -3763,7 +3756,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H4" s="2">
         <v>7.2</v>
@@ -3787,16 +3780,16 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="C5" s="2">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" s="2">
         <v>12.5</v>
@@ -3805,7 +3798,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H5" s="2">
         <v>14</v>
@@ -3829,16 +3822,16 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="C6" s="2">
         <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2">
         <v>34</v>
@@ -3847,7 +3840,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H6" s="2">
         <v>31</v>
@@ -3871,16 +3864,16 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="C7" s="2">
         <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" s="2">
         <v>2.5</v>
@@ -3889,7 +3882,7 @@
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H7" s="2">
         <v>2.8</v>
@@ -3913,16 +3906,16 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="C8" s="2">
         <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E8" s="2">
         <v>4.2</v>
@@ -3931,7 +3924,7 @@
         <v>18</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H8" s="2">
         <v>3.9</v>
@@ -3955,16 +3948,16 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2">
         <v>280</v>
@@ -3973,7 +3966,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H9" s="2">
         <v>265</v>
@@ -3997,16 +3990,16 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="2">
         <v>45</v>
@@ -4015,7 +4008,7 @@
         <v>22</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H10" s="2">
         <v>48</v>
@@ -4039,16 +4032,16 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11" s="2">
         <v>32</v>
@@ -4057,7 +4050,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H11" s="2">
         <v>29</v>

</xml_diff>

<commit_message>
Fix cotacao totals to use qty times unit price plus freight.
The grader previously ignored quantity; Melhor now also accepts the cheaper supplier name.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/exercicios/treino-compras-01-cotacao.xlsx
+++ b/public/exercicios/treino-compras-01-cotacao.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="62">
   <si>
     <t>TREINO COMPRAS — Exercício 1: Cotação</t>
   </si>
@@ -31,13 +31,13 @@
     <t>2) Nas células AMARELAS, digite fórmulas (não copie números na mão)</t>
   </si>
   <si>
-    <t>3) Coluna J (Total1): =E2+F2  e arraste até a linha 11</t>
-  </si>
-  <si>
-    <t>4) Coluna K (Total2): =H2+I2  e arraste até a linha 11</t>
-  </si>
-  <si>
-    <t>5) Coluna L (Melhor): =MÍNIMO(J2:K2)  ou  =MIN(J2:K2)</t>
+    <t>3) Coluna J (Total1): =C2*E2+F2  (Qtd × Preço1 + Frete1) e arraste até a linha 11</t>
+  </si>
+  <si>
+    <t>4) Coluna K (Total2): =C2*H2+I2  (Qtd × Preço2 + Frete2) e arraste até a linha 11</t>
+  </si>
+  <si>
+    <t>5) Coluna L (Melhor): =MÍNIMO(J2:K2)  ou  =MIN(J2:K2)  — o menor TOTAL (número)</t>
   </si>
   <si>
     <t>6) Se abriu só em visualização, use Editar no navegador / Salvar uma cópia</t>
@@ -178,19 +178,25 @@
     <t>J2</t>
   </si>
   <si>
-    <t>=E2+F2</t>
+    <t>=C2*E2+F2</t>
   </si>
   <si>
     <t>K2</t>
   </si>
   <si>
-    <t>=H2+I2</t>
+    <t>=C2*H2+I2</t>
   </si>
   <si>
     <t>L2</t>
   </si>
   <si>
     <t>=MIN(J2:K2)   (no Excel PT-BR também pode =MÍNIMO(J2:K2))</t>
+  </si>
+  <si>
+    <t>Total = quantidade × preço unitário + frete.</t>
+  </si>
+  <si>
+    <t>Melhor = menor total (número), não o nome do fornecedor.</t>
   </si>
   <si>
     <t>Não abra a aba Gabarito antes de tentar.</t>
@@ -2808,7 +2814,9 @@
       <c r="P6" s="2"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2826,7 +2834,9 @@
       <c r="P7" s="2"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
+      <c r="A8" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -3681,13 +3691,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="2">
-        <v>25.95</v>
+        <v>120</v>
       </c>
       <c r="K2" s="2">
-        <v>1.1</v>
+        <v>110</v>
       </c>
       <c r="L2" s="2">
-        <v>1.1</v>
+        <v>110</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -3723,13 +3733,13 @@
         <v>20</v>
       </c>
       <c r="J3" s="2">
-        <v>15.18</v>
+        <v>33</v>
       </c>
       <c r="K3" s="2">
-        <v>20.15</v>
+        <v>35</v>
       </c>
       <c r="L3" s="2">
-        <v>15.18</v>
+        <v>33</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -3765,13 +3775,13 @@
         <v>80</v>
       </c>
       <c r="J4" s="2">
-        <v>38</v>
+        <v>430</v>
       </c>
       <c r="K4" s="2">
-        <v>87.2</v>
+        <v>440</v>
       </c>
       <c r="L4" s="2">
-        <v>38</v>
+        <v>430</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -3807,13 +3817,13 @@
         <v>0</v>
       </c>
       <c r="J5" s="2">
-        <v>32.5</v>
+        <v>145</v>
       </c>
       <c r="K5" s="2">
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="L5" s="2">
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -3849,13 +3859,13 @@
         <v>90</v>
       </c>
       <c r="J6" s="2">
-        <v>79</v>
+        <v>725</v>
       </c>
       <c r="K6" s="2">
-        <v>121</v>
+        <v>710</v>
       </c>
       <c r="L6" s="2">
-        <v>79</v>
+        <v>710</v>
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -3891,13 +3901,13 @@
         <v>0</v>
       </c>
       <c r="J7" s="2">
-        <v>17.5</v>
+        <v>65</v>
       </c>
       <c r="K7" s="2">
-        <v>2.8</v>
+        <v>56</v>
       </c>
       <c r="L7" s="2">
-        <v>2.8</v>
+        <v>56</v>
       </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -3933,13 +3943,13 @@
         <v>25</v>
       </c>
       <c r="J8" s="2">
-        <v>22.2</v>
+        <v>123</v>
       </c>
       <c r="K8" s="2">
-        <v>28.9</v>
+        <v>122.5</v>
       </c>
       <c r="L8" s="2">
-        <v>22.2</v>
+        <v>122.5</v>
       </c>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -4017,13 +4027,13 @@
         <v>0</v>
       </c>
       <c r="J10" s="2">
-        <v>67</v>
+        <v>247</v>
       </c>
       <c r="K10" s="2">
-        <v>48</v>
+        <v>240</v>
       </c>
       <c r="L10" s="2">
-        <v>48</v>
+        <v>240</v>
       </c>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -4059,13 +4069,13 @@
         <v>35</v>
       </c>
       <c r="J11" s="2">
-        <v>60</v>
+        <v>220</v>
       </c>
       <c r="K11" s="2">
-        <v>64</v>
+        <v>209</v>
       </c>
       <c r="L11" s="2">
-        <v>60</v>
+        <v>209</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>

</xml_diff>

<commit_message>
Teach Empate with nested SE and add two new Excel drills.
Decision and quote exercises now write Empate on ties; new packs cover prazo tie-break and three-supplier CONT.SE logic.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/exercicios/treino-compras-01-cotacao.xlsx
+++ b/public/exercicios/treino-compras-01-cotacao.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="64">
   <si>
     <t>TREINO COMPRAS — Exercício 1: Cotação</t>
   </si>
@@ -37,7 +37,10 @@
     <t>4) Coluna K (Total2): =C2*H2+I2  (Qtd × Preço2 + Frete2) e arraste até a linha 11</t>
   </si>
   <si>
-    <t>5) Coluna L (Melhor): =MÍNIMO(J2:K2)  ou  =MIN(J2:K2)  — o menor TOTAL (número)</t>
+    <t>5) Coluna L (Melhor): =SE(J2=K2;"Empate";SE(J2&lt;K2;D2;G2))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   → mostra o fornecedor mais barato OU a palavra Empate</t>
   </si>
   <si>
     <t>6) Se abriu só em visualização, use Editar no navegador / Salvar uma cópia</t>
@@ -190,16 +193,19 @@
     <t>L2</t>
   </si>
   <si>
-    <t>=MIN(J2:K2)   (no Excel PT-BR também pode =MÍNIMO(J2:K2))</t>
+    <t>=SE(J2=K2;"Empate";SE(J2&lt;K2;D2;G2))</t>
   </si>
   <si>
     <t>Total = quantidade × preço unitário + frete.</t>
   </si>
   <si>
-    <t>Melhor = menor total (número), não o nome do fornecedor.</t>
+    <t>Se Total1 = Total2, a fórmula deve escrever Empate (não escolher um lado).</t>
   </si>
   <si>
     <t>Não abra a aba Gabarito antes de tentar.</t>
+  </si>
+  <si>
+    <t>Empate</t>
   </si>
 </sst>
 </file>
@@ -829,7 +835,9 @@
       <c r="P10" s="2"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -1570,40 +1578,40 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
@@ -1612,16 +1620,16 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2">
         <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2">
         <v>0.95</v>
@@ -1630,7 +1638,7 @@
         <v>25</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H2" s="2">
         <v>1.1</v>
@@ -1648,16 +1656,16 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2">
         <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2">
         <v>0.18</v>
@@ -1666,7 +1674,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H3" s="2">
         <v>0.15</v>
@@ -1684,16 +1692,16 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2">
         <v>50</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="2">
         <v>8</v>
@@ -1702,7 +1710,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="2">
         <v>7.2</v>
@@ -1720,16 +1728,16 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="2">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" s="2">
         <v>12.5</v>
@@ -1738,7 +1746,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H5" s="2">
         <v>14</v>
@@ -1756,16 +1764,16 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="2">
         <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" s="2">
         <v>34</v>
@@ -1774,7 +1782,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H6" s="2">
         <v>31</v>
@@ -1792,16 +1800,16 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="2">
         <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" s="2">
         <v>2.5</v>
@@ -1810,7 +1818,7 @@
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2">
         <v>2.8</v>
@@ -1828,16 +1836,16 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2">
         <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E8" s="2">
         <v>4.2</v>
@@ -1846,7 +1854,7 @@
         <v>18</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H8" s="2">
         <v>3.9</v>
@@ -1864,16 +1872,16 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" s="2">
         <v>280</v>
@@ -1882,7 +1890,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H9" s="2">
         <v>265</v>
@@ -1900,16 +1908,16 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10" s="2">
         <v>45</v>
@@ -1918,7 +1926,7 @@
         <v>22</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H10" s="2">
         <v>48</v>
@@ -1936,16 +1944,16 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E11" s="2">
         <v>32</v>
@@ -1954,7 +1962,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H11" s="2">
         <v>29</v>
@@ -2689,7 +2697,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2709,10 +2717,10 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2731,10 +2739,10 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -2753,10 +2761,10 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2795,7 +2803,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -2815,7 +2823,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2835,7 +2843,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -3622,40 +3630,40 @@
   <sheetData>
     <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
@@ -3664,16 +3672,16 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2">
         <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2">
         <v>0.95</v>
@@ -3682,7 +3690,7 @@
         <v>25</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H2" s="2">
         <v>1.1</v>
@@ -3696,8 +3704,8 @@
       <c r="K2" s="2">
         <v>110</v>
       </c>
-      <c r="L2" s="2">
-        <v>110</v>
+      <c r="L2" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -3706,16 +3714,16 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2">
         <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2">
         <v>0.18</v>
@@ -3724,7 +3732,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H3" s="2">
         <v>0.15</v>
@@ -3738,8 +3746,8 @@
       <c r="K3" s="2">
         <v>35</v>
       </c>
-      <c r="L3" s="2">
-        <v>33</v>
+      <c r="L3" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -3748,16 +3756,16 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2">
         <v>50</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="2">
         <v>8</v>
@@ -3766,7 +3774,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="2">
         <v>7.2</v>
@@ -3780,8 +3788,8 @@
       <c r="K4" s="2">
         <v>440</v>
       </c>
-      <c r="L4" s="2">
-        <v>430</v>
+      <c r="L4" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -3790,16 +3798,16 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="2">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" s="2">
         <v>12.5</v>
@@ -3808,7 +3816,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H5" s="2">
         <v>14</v>
@@ -3822,8 +3830,8 @@
       <c r="K5" s="2">
         <v>140</v>
       </c>
-      <c r="L5" s="2">
-        <v>140</v>
+      <c r="L5" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -3832,16 +3840,16 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="2">
         <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" s="2">
         <v>34</v>
@@ -3850,7 +3858,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H6" s="2">
         <v>31</v>
@@ -3864,8 +3872,8 @@
       <c r="K6" s="2">
         <v>710</v>
       </c>
-      <c r="L6" s="2">
-        <v>710</v>
+      <c r="L6" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -3874,16 +3882,16 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="2">
         <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" s="2">
         <v>2.5</v>
@@ -3892,7 +3900,7 @@
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2">
         <v>2.8</v>
@@ -3906,8 +3914,8 @@
       <c r="K7" s="2">
         <v>56</v>
       </c>
-      <c r="L7" s="2">
-        <v>56</v>
+      <c r="L7" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -3916,16 +3924,16 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2">
         <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E8" s="2">
         <v>4.2</v>
@@ -3934,7 +3942,7 @@
         <v>18</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H8" s="2">
         <v>3.9</v>
@@ -3948,8 +3956,8 @@
       <c r="K8" s="2">
         <v>122.5</v>
       </c>
-      <c r="L8" s="2">
-        <v>122.5</v>
+      <c r="L8" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -3958,16 +3966,16 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" s="2">
         <v>280</v>
@@ -3976,7 +3984,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H9" s="2">
         <v>265</v>
@@ -3990,8 +3998,8 @@
       <c r="K9" s="2">
         <v>320</v>
       </c>
-      <c r="L9" s="2">
-        <v>320</v>
+      <c r="L9" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -4000,16 +4008,16 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10" s="2">
         <v>45</v>
@@ -4018,7 +4026,7 @@
         <v>22</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H10" s="2">
         <v>48</v>
@@ -4032,8 +4040,8 @@
       <c r="K10" s="2">
         <v>240</v>
       </c>
-      <c r="L10" s="2">
-        <v>240</v>
+      <c r="L10" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -4042,16 +4050,16 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E11" s="2">
         <v>32</v>
@@ -4060,7 +4068,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H11" s="2">
         <v>29</v>
@@ -4074,8 +4082,8 @@
       <c r="K11" s="2">
         <v>209</v>
       </c>
-      <c r="L11" s="2">
-        <v>209</v>
+      <c r="L11" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>

</xml_diff>